<commit_message>
Nytt premium-design, Excel-oppgaver live i nettleseren og jevne animasjoner
- Svart-hvitt design med Geist / Geist Mono, uten gradienter
- Oppgaver-fanen kjører Excel-arkene med HyperFormula (samme formler som xlsx)
- Rullende avsløringer, glidende faner, sideoverganger og Lenis-scroll
- KVR-diagram med dekningspunkt og hover
- verktoy/xlsx_til_json.py eksporterer Excel-filen til nettsiden

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eksempler/HSM122_eksempeloppgaver.xlsx
+++ b/eksempler/HSM122_eksempeloppgaver.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bendi\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8318DA3B-409C-40AB-9BB8-5E2431D58B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D1786F-E2A1-4408-9B2D-5A4AD21A98B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1851" yWindow="1851" windowWidth="22115" windowHeight="8400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="353">
   <si>
     <t>HSM122 – Eksempeloppgaver</t>
   </si>
@@ -858,6 +858,9 @@
   </si>
   <si>
     <t>B) Standardkost – inndata</t>
+  </si>
+  <si>
+    <t>Formel / merknad</t>
   </si>
   <si>
     <t>Produserte enheter</t>
@@ -1439,7 +1442,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3A20-40EB-985E-4C0B50544135}"/>
+              <c16:uniqueId val="{00000000-05C8-4790-B30B-DD677E646D9C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1543,7 +1546,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3A20-40EB-985E-4C0B50544135}"/>
+              <c16:uniqueId val="{00000001-05C8-4790-B30B-DD677E646D9C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1647,7 +1650,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3A20-40EB-985E-4C0B50544135}"/>
+              <c16:uniqueId val="{00000002-05C8-4790-B30B-DD677E646D9C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5241,15 +5244,15 @@
         <v>232</v>
       </c>
       <c r="B18" s="33">
-        <f>RANK(B17,$B$17:$D$17)</f>
+        <f>1+COUNTIF($B$17:$D$17,"&gt;"&amp;B17)</f>
         <v>3</v>
       </c>
       <c r="C18" s="33">
-        <f>RANK(C17,$B$17:$D$17)</f>
+        <f>1+COUNTIF($B$17:$D$17,"&gt;"&amp;C17)</f>
         <v>1</v>
       </c>
       <c r="D18" s="33">
-        <f>RANK(D17,$B$17:$D$17)</f>
+        <f>1+COUNTIF($B$17:$D$17,"&gt;"&amp;D17)</f>
         <v>2</v>
       </c>
       <c r="E18" s="17" t="s">
@@ -5299,15 +5302,15 @@
         <v>237</v>
       </c>
       <c r="B21" s="33">
-        <f>SUMPRODUCT(($B$18:$D$18&lt;B18)*$B$20:$D$20)</f>
+        <f>SUMIF($B$18:$D$18,"&lt;"&amp;B18,$B$20:$D$20)</f>
         <v>9000</v>
       </c>
       <c r="C21" s="33">
-        <f>SUMPRODUCT(($B$18:$D$18&lt;C18)*$B$20:$D$20)</f>
+        <f>SUMIF($B$18:$D$18,"&lt;"&amp;C18,$B$20:$D$20)</f>
         <v>0</v>
       </c>
       <c r="D21" s="33">
-        <f>SUMPRODUCT(($B$18:$D$18&lt;D18)*$B$20:$D$20)</f>
+        <f>SUMIF($B$18:$D$18,"&lt;"&amp;D18,$B$20:$D$20)</f>
         <v>4000</v>
       </c>
       <c r="E21" s="17"/>
@@ -5681,14 +5684,13 @@
       <c r="B20" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13" t="s">
-        <v>78</v>
+      <c r="C20" s="13" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="8" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B21" s="22">
         <v>1000</v>
@@ -5701,7 +5703,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A22" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B22" s="22">
         <v>4</v>
@@ -5714,7 +5716,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A23" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B23" s="14">
         <v>25</v>
@@ -5727,7 +5729,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A24" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B24" s="22">
         <v>4300</v>
@@ -5740,7 +5742,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A25" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B25" s="14">
         <v>24</v>
@@ -5753,7 +5755,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A26" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B26" s="22">
         <v>2</v>
@@ -5766,7 +5768,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A27" s="8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B27" s="14">
         <v>300</v>
@@ -5779,7 +5781,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A28" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B28" s="22">
         <v>2100</v>
@@ -5792,7 +5794,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A29" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B29" s="14">
         <v>310</v>
@@ -5805,7 +5807,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A30" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B30" s="14">
         <v>80</v>
@@ -5818,7 +5820,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A31" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B31" s="14">
         <v>175000</v>
@@ -5831,7 +5833,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A32" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B32" s="14">
         <v>240000</v>
@@ -5844,7 +5846,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A33" s="8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B33" s="22">
         <v>2400</v>
@@ -5857,7 +5859,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A34" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B34" s="14">
         <v>250000</v>
@@ -5870,14 +5872,14 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A35" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B35" s="33">
         <f>$B$22*$B$21</f>
         <v>4000</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8"/>
@@ -5886,14 +5888,14 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A36" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B36" s="33">
         <f>$B$26*$B$21</f>
         <v>2000</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
@@ -5902,14 +5904,14 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A37" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B37" s="16">
         <f>$B$32/$B$33</f>
         <v>100</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
@@ -5918,14 +5920,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A38" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B38" s="16">
         <f>$B$22*$B$23+$B$26*$B$27+$B$26*($B$30+$B$37)</f>
         <v>1060</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D38" s="8"/>
       <c r="E38" s="8"/>
@@ -5934,7 +5936,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B40" s="12"/>
       <c r="C40" s="12"/>
@@ -5954,17 +5956,17 @@
         <v>249</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A42" s="35" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A43" s="8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B43" s="16">
         <f>($B$23-$B$25)*$B$24</f>
@@ -5975,7 +5977,7 @@
         <v>Gunstig</v>
       </c>
       <c r="D43" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E43" s="8"/>
       <c r="F43" s="8"/>
@@ -5983,7 +5985,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A44" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B44" s="16">
         <f>($B$35-$B$24)*$B$23</f>
@@ -5994,7 +5996,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D44" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E44" s="8"/>
       <c r="F44" s="8"/>
@@ -6002,7 +6004,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A45" s="19" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B45" s="21">
         <f>$B$43+$B$44</f>
@@ -6013,7 +6015,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D45" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E45" s="8"/>
       <c r="F45" s="8"/>
@@ -6021,14 +6023,14 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A46" s="8" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B46" s="16">
         <f>$B$35*$B$23-$B$24*$B$25</f>
         <v>-3200</v>
       </c>
       <c r="C46" s="17" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="8"/>
@@ -6037,12 +6039,12 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A47" s="35" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A48" s="8" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B48" s="16">
         <f>($B$27-$B$29)*$B$28</f>
@@ -6053,7 +6055,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D48" s="17" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E48" s="8"/>
       <c r="F48" s="8"/>
@@ -6061,7 +6063,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A49" s="8" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B49" s="16">
         <f>($B$36-$B$28)*$B$27</f>
@@ -6072,7 +6074,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D49" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E49" s="8"/>
       <c r="F49" s="8"/>
@@ -6080,7 +6082,7 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A50" s="19" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B50" s="21">
         <f>$B$36*$B$27-$B$28*$B$29</f>
@@ -6091,7 +6093,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E50" s="8"/>
       <c r="F50" s="8"/>
@@ -6099,12 +6101,12 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A51" s="35" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A52" s="8" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B52" s="16">
         <f>$B$28*$B$30-$B$31</f>
@@ -6115,7 +6117,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D52" s="17" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E52" s="8"/>
       <c r="F52" s="8"/>
@@ -6123,7 +6125,7 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A53" s="8" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B53" s="16">
         <f>$B$36*$B$30-$B$28*$B$30</f>
@@ -6134,7 +6136,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D53" s="17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E53" s="8"/>
       <c r="F53" s="8"/>
@@ -6142,7 +6144,7 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A54" s="19" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B54" s="21">
         <f>$B$52+$B$53</f>
@@ -6159,12 +6161,12 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A55" s="35" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A56" s="8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B56" s="16">
         <f>$B$32-$B$34</f>
@@ -6175,7 +6177,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E56" s="8"/>
       <c r="F56" s="8"/>
@@ -6183,7 +6185,7 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A57" s="8" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B57" s="16">
         <f>$B$36*$B$37-$B$32</f>
@@ -6194,7 +6196,7 @@
         <v>Ugunstig</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E57" s="8"/>
       <c r="F57" s="8"/>
@@ -6202,7 +6204,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A58" s="19" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B58" s="21">
         <f>$B$56+$B$57</f>
@@ -6239,7 +6241,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="9" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.4">
@@ -6249,7 +6251,7 @@
     </row>
     <row r="4" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="37" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B4" s="38"/>
       <c r="C4" s="38"/>
@@ -6260,7 +6262,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
@@ -6272,18 +6274,18 @@
     <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="13"/>
       <c r="B7" s="13" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B8" s="14">
         <v>300000</v>
@@ -6295,7 +6297,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B9" s="22">
         <v>2000</v>
@@ -6307,7 +6309,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="8" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B10" s="22">
         <v>1800</v>
@@ -6319,7 +6321,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="8" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B11" s="22">
         <v>1850</v>
@@ -6331,7 +6333,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B12" s="22">
         <v>1900</v>
@@ -6343,7 +6345,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="8" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B13" s="14">
         <v>310000</v>
@@ -6355,7 +6357,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="19" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B14" s="20">
         <f>B8/B9</f>
@@ -6366,12 +6368,12 @@
         <v>500</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="8" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B15" s="16">
         <f>(B10-B9)*B14</f>
@@ -6382,12 +6384,12 @@
         <v>-10000</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="8" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B16" s="16">
         <f>(B11-B12)*B14</f>
@@ -6398,12 +6400,12 @@
         <v>-15000</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A17" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B17" s="16">
         <f>B8-B13</f>
@@ -6414,12 +6416,12 @@
         <v>4000</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A18" s="8" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B18" s="16">
         <f>(B12-B9)*B14</f>
@@ -6430,17 +6432,17 @@
         <v>-5000</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A21" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -6451,16 +6453,16 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A22" s="13" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>141</v>
@@ -6468,7 +6470,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A23" s="34" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B23" s="22">
         <v>1200</v>
@@ -6481,12 +6483,12 @@
         <v>255000</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A24" s="34" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B24" s="22">
         <v>700</v>
@@ -6499,12 +6501,12 @@
         <v>225000</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A25" s="34" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B25" s="26">
         <f>SUM(B23:B24)</f>
@@ -6519,7 +6521,7 @@
         <v>480000</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>